<commit_message>
added upload photo function
</commit_message>
<xml_diff>
--- a/incomes_details.xlsx
+++ b/incomes_details.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,51 +413,18 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Youtube</v>
+        <v>salary</v>
       </c>
       <c r="B2">
-        <v>9500</v>
+        <v>50000</v>
       </c>
       <c r="C2" s="1">
-        <v>45825.291712962964</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Trading</v>
-      </c>
-      <c r="B3">
-        <v>10000</v>
-      </c>
-      <c r="C3" s="1">
-        <v>45823.291712962964</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Business</v>
-      </c>
-      <c r="B4">
-        <v>6500</v>
-      </c>
-      <c r="C4" s="1">
-        <v>45820.291712962964</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Salary</v>
-      </c>
-      <c r="B5">
-        <v>12500</v>
-      </c>
-      <c r="C5" s="1">
-        <v>45809.291712962964</v>
+        <v>45901.291712962964</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>